<commit_message>
Update: Bo sung Sheet 8 cong cu AI cho kenh Ke Chuyen day ky nang cho be
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KeHoach_KenhYT_KeChuyen.xlsx
+++ b/KeHoach_KenhYT_KeChuyen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00114129-FE1F-4C2B-BDC8-C4046E8C73F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54610A7E-2CE4-4A69-8B54-035569101A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="6" xr2:uid="{09AEB785-3603-4D50-A6FD-8B8A6EC4BE27}"/>
+    <workbookView xWindow="-4125" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{B0484EF4-63C2-4983-9CEB-04CD81028A15}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Tong Quan" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="5. KPIs Theo Doi" sheetId="5" r:id="rId5"/>
     <sheet name="6. Quy Trinh" sheetId="6" r:id="rId6"/>
     <sheet name="7. Chi Tiet Series" sheetId="7" r:id="rId7"/>
+    <sheet name="8. Cong Cu AI" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="617">
   <si>
     <t>KE HOACH KENH YOUTUBE - KE CHUYEN DAY KY NANG SONG CHO BE</t>
   </si>
@@ -1467,18 +1468,448 @@
   </si>
   <si>
     <t>Khong chia se thong tin ca nhan online</t>
+  </si>
+  <si>
+    <t>CONG CU AI CHO KENH KE CHUYEN - DAY KY NANG SONG CHO BE</t>
+  </si>
+  <si>
+    <t>Giai Doan San Xuat</t>
+  </si>
+  <si>
+    <t>Cong Cu AI</t>
+  </si>
+  <si>
+    <t>Chuc Nang Cu The</t>
+  </si>
+  <si>
+    <t>Muc Gia</t>
+  </si>
+  <si>
+    <t>Muc Do Uu Tien</t>
+  </si>
+  <si>
+    <t>Luu Y</t>
+  </si>
+  <si>
+    <t>BUOC 1: VIET KICH BAN &amp; Y TUONG</t>
+  </si>
+  <si>
+    <t>Viet kich ban chuyen</t>
+  </si>
+  <si>
+    <t>ChatGPT / Claude</t>
+  </si>
+  <si>
+    <t>Prompt: 'Viet kich ban ke chuyen ve ky nang [X] cho be 5 tuoi, co nhan vat de thuong, tinh huong thuc te, thong diep ro rang'</t>
+  </si>
+  <si>
+    <t>Mien phi / /thang</t>
+  </si>
+  <si>
+    <t>CAO NHAT</t>
+  </si>
+  <si>
+    <t>Claude rat tot cho van ban Viet</t>
+  </si>
+  <si>
+    <t>Brainstorm y tuong</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Goi y chuyen theo chu de ky nang song, phu hop vung mien VN</t>
+  </si>
+  <si>
+    <t>Mien phi</t>
+  </si>
+  <si>
+    <t>CAO</t>
+  </si>
+  <si>
+    <t>Hieu van hoa Viet tot</t>
+  </si>
+  <si>
+    <t>SEO tieu de video</t>
+  </si>
+  <si>
+    <t>ChatGPT + TubeBuddy AI</t>
+  </si>
+  <si>
+    <t>Tim tu khoa phu huynh hay tim khi cho be xem: 'chuyen be...', 'day be...'</t>
+  </si>
+  <si>
+    <t>/thang (TB)</t>
+  </si>
+  <si>
+    <t>TRUNG BINH</t>
+  </si>
+  <si>
+    <t>Ket hop 2 cong cu</t>
+  </si>
+  <si>
+    <t>BUOC 2: TAO HINH ANH &amp; NHAN VAT</t>
+  </si>
+  <si>
+    <t>Tao nhan vat chinh</t>
+  </si>
+  <si>
+    <t>Midjourney v6</t>
+  </si>
+  <si>
+    <t>Prompt: 'cute Vietnamese cartoon child character, simple, friendly, 2D flat design, Pixar style'</t>
+  </si>
+  <si>
+    <t>/thang</t>
+  </si>
+  <si>
+    <t>Nhat quan bo nhan vat</t>
+  </si>
+  <si>
+    <t>Ve background / canh</t>
+  </si>
+  <si>
+    <t>DALL-E 3 (ChatGPT)</t>
+  </si>
+  <si>
+    <t>Tao canh: truong hoc, gia dinh, san choi Viet Nam phong cach cartoon</t>
+  </si>
+  <si>
+    <t>Mien phi (co han)</t>
+  </si>
+  <si>
+    <t>Mien phi trong ChatGPT Plus</t>
+  </si>
+  <si>
+    <t>Chinh sua &amp; ghep hinh</t>
+  </si>
+  <si>
+    <t>Adobe Firefly</t>
+  </si>
+  <si>
+    <t>Xoa nen, thay doi mau sac nhan vat, chuan hoa phong cach</t>
+  </si>
+  <si>
+    <t>Free / /thang</t>
+  </si>
+  <si>
+    <t>Tich hop san trong Adobe</t>
+  </si>
+  <si>
+    <t>Thiet ke nhanh</t>
+  </si>
+  <si>
+    <t>Canva AI (Magic Design)</t>
+  </si>
+  <si>
+    <t>Tao thumbnail, poster, banner kenh tu text prompt</t>
+  </si>
+  <si>
+    <t>De dung nhat cho nguoi moi</t>
+  </si>
+  <si>
+    <t>BUOC 3: GIONG DOC &amp; AM THANH</t>
+  </si>
+  <si>
+    <t>Giong ke chuyen tieng Viet</t>
+  </si>
+  <si>
+    <t>FPT.AI Voice</t>
+  </si>
+  <si>
+    <t>Text-to-speech tieng Viet nhieu giong (Nam Bac, giong nu/nam, giong tre em)</t>
+  </si>
+  <si>
+    <t>Mien phi co han</t>
+  </si>
+  <si>
+    <t>Tieng Viet tu nhien nhat</t>
+  </si>
+  <si>
+    <t>Giong doc chat luong cao</t>
+  </si>
+  <si>
+    <t>ElevenLabs</t>
+  </si>
+  <si>
+    <t>Clone giong hoac dung giong san, rat tu nhien, ho tro tieng Viet</t>
+  </si>
+  <si>
+    <t>-22/thang</t>
+  </si>
+  <si>
+    <t>Chat luong tot nhat hien tai</t>
+  </si>
+  <si>
+    <t>Backup giong doc</t>
+  </si>
+  <si>
+    <t>Murf AI</t>
+  </si>
+  <si>
+    <t>Thu vien giong da dang, co tieng Viet co ban</t>
+  </si>
+  <si>
+    <t>Goi y neu ElevenLabs dat</t>
+  </si>
+  <si>
+    <t>Tao nhac nen thieu nhi</t>
+  </si>
+  <si>
+    <t>Suno AI</t>
+  </si>
+  <si>
+    <t>Prompt: 'happy children background music, ukulele, soft, Vietnamese style, no lyrics'</t>
+  </si>
+  <si>
+    <t>Nhac doc quyen, khong copyright</t>
+  </si>
+  <si>
+    <t>Tao nhac nen 2</t>
+  </si>
+  <si>
+    <t>Udio</t>
+  </si>
+  <si>
+    <t>Tuong tu Suno, them tuy chon nhac cu, nhac dan toc</t>
+  </si>
+  <si>
+    <t>Mien phi beta</t>
+  </si>
+  <si>
+    <t>Dang trong giai doan beta</t>
+  </si>
+  <si>
+    <t>BUOC 4: LAM HOAT HINH &amp; VIDEO</t>
+  </si>
+  <si>
+    <t>Lam hoat hinh slide 2D</t>
+  </si>
+  <si>
+    <t>Animaker AI</t>
+  </si>
+  <si>
+    <t>Keo tha nhan vat, them dong tac, phong cach cartoon dep cho be</t>
+  </si>
+  <si>
+    <t>-20/thang</t>
+  </si>
+  <si>
+    <t>De dung, nhieu template thieu nhi</t>
+  </si>
+  <si>
+    <t>Tao video tu hinh anh</t>
+  </si>
+  <si>
+    <t>Kling AI (Kuaishou)</t>
+  </si>
+  <si>
+    <t>Bien hinh anh nhan vat thanh video co chuyen dong tu nhien</t>
+  </si>
+  <si>
+    <t>Chuyen dong rat dep</t>
+  </si>
+  <si>
+    <t>Chinh sua video AI</t>
+  </si>
+  <si>
+    <t>CapCut AI</t>
+  </si>
+  <si>
+    <t>Tu dong cat ghep, them phu de, hieu ung, chinh mau sac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mien phi / Pro </t>
+  </si>
+  <si>
+    <t>De dung, nhieu template VN</t>
+  </si>
+  <si>
+    <t>Hieu ung chuyen canh</t>
+  </si>
+  <si>
+    <t>Runway ML</t>
+  </si>
+  <si>
+    <t>Tao hieu ung bien doi canh dep, hieu ung dac biet</t>
+  </si>
+  <si>
+    <t>Dung cho canh dac biet</t>
+  </si>
+  <si>
+    <t>Avatar nguoi ke chuyen</t>
+  </si>
+  <si>
+    <t>HeyGen</t>
+  </si>
+  <si>
+    <t>Tao avatar AI ke chuyen that, dong bo moi voi giong doc</t>
+  </si>
+  <si>
+    <t>Neu muon co nguoi that dong</t>
+  </si>
+  <si>
+    <t>BUOC 5: PHAN DE &amp; BIEN TAP</t>
+  </si>
+  <si>
+    <t>Tu dong tao phu de</t>
+  </si>
+  <si>
+    <t>Kapwing AI</t>
+  </si>
+  <si>
+    <t>Upload video, AI tu dong tao phu de tieng Viet chinh xac</t>
+  </si>
+  <si>
+    <t>Giup be theo doi dung hon</t>
+  </si>
+  <si>
+    <t>Chinh sua phu de</t>
+  </si>
+  <si>
+    <t>Descript</t>
+  </si>
+  <si>
+    <t>Sua phu de nhu sua van ban, cat video bang cach xoa chu</t>
+  </si>
+  <si>
+    <t>Rat thuan tien cho bien tap</t>
+  </si>
+  <si>
+    <t>Kiem tra noi dung an toan</t>
+  </si>
+  <si>
+    <t>YouTube Safety Check</t>
+  </si>
+  <si>
+    <t>Xem lai nguon: YouTube chay Content ID tu dong</t>
+  </si>
+  <si>
+    <t>BAT BUOC</t>
+  </si>
+  <si>
+    <t>Tranh copyright nhac, hinh</t>
+  </si>
+  <si>
+    <t>BUOC 6: DANG VIDEO &amp; SEO</t>
+  </si>
+  <si>
+    <t>Toi uu SEO YouTube</t>
+  </si>
+  <si>
+    <t>VidIQ AI (Boost)</t>
+  </si>
+  <si>
+    <t>Phan tich tu khoa, goi y tieu de/tag, xem score SEO</t>
+  </si>
+  <si>
+    <t>Plugin Chrome de cai</t>
+  </si>
+  <si>
+    <t>Toi uu SEO bo sung</t>
+  </si>
+  <si>
+    <t>TubeBuddy AI</t>
+  </si>
+  <si>
+    <t>A/B test thumbnail, tag explorer, best time to post</t>
+  </si>
+  <si>
+    <t>Ket hop voi VidIQ</t>
+  </si>
+  <si>
+    <t>Tao thumbnail hap dan</t>
+  </si>
+  <si>
+    <t>Canva AI + Magic Write</t>
+  </si>
+  <si>
+    <t>Tao thumbnail: nhan vat chinh + chu ngan gon + mau sac noi bat</t>
+  </si>
+  <si>
+    <t>Font chu lon &gt; 40pt</t>
+  </si>
+  <si>
+    <t>Viet mo ta video</t>
+  </si>
+  <si>
+    <t>Claude / ChatGPT</t>
+  </si>
+  <si>
+    <t>Viet mo ta 200-500 chu, co tu khoa, goi y xem them video khac</t>
+  </si>
+  <si>
+    <t>Nen dung template co san</t>
+  </si>
+  <si>
+    <t>BUOC 7: PHAN TICH &amp; PHAT TRIEN</t>
+  </si>
+  <si>
+    <t>Phan tich hieu suat</t>
+  </si>
+  <si>
+    <t>YouTube Analytics + AI</t>
+  </si>
+  <si>
+    <t>Xem CTR, watch time, tuoi nguoi xem theo doi tu dong</t>
+  </si>
+  <si>
+    <t>Xem moi tuan 1 lan</t>
+  </si>
+  <si>
+    <t>Hieu content de tang view</t>
+  </si>
+  <si>
+    <t>Opus Clip AI</t>
+  </si>
+  <si>
+    <t>Tu dong cat clip ngan viral tu video dai, dang TikTok/Reels</t>
+  </si>
+  <si>
+    <t>Tang traffic tu TikTok ve YT</t>
+  </si>
+  <si>
+    <t>Quan ly lich dang</t>
+  </si>
+  <si>
+    <t>Buffer AI Assist</t>
+  </si>
+  <si>
+    <t>Lap lich dang nhieu kenh, goi y gio vang, theo doi tuong tac</t>
+  </si>
+  <si>
+    <t>Quan ly FB, TikTok, YT 1 cho</t>
+  </si>
+  <si>
+    <t>Nghien cuu doi thu</t>
+  </si>
+  <si>
+    <t>ChatGPT + YouTube</t>
+  </si>
+  <si>
+    <t>Phan tich kenh ke chuyen lon (Peppa Pig VN, Thoi Gian Vang...)</t>
+  </si>
+  <si>
+    <t>Hoc tu kenh thanh cong</t>
+  </si>
+  <si>
+    <t>AI STACK TIEU CHUAN DE XUAT (chi phi ~500K-1.5 trieu VND/thang): FPT.AI Voice + Midjourney + Animaker + CapCut AI + VidIQ + Suno AI + ChatGPT/Claude</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#.##0"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="163"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1534,10 +1965,27 @@
       <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="32">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1694,6 +2142,36 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF366B1F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF50B000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF66D9FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1722,7 +2200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1782,12 +2260,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1880,6 +2358,69 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2213,34 +2754,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17170A6E-FC07-4B91-A7A6-A07CE076B7FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D04617F3-6085-4A85-97CB-EDAA1E473E8B}">
   <sheetPr>
     <tabColor rgb="FF9D6BFF"/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" customWidth="1"/>
+    <col min="2" max="2" width="50.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="50.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" s="4"/>
       <c r="B2" s="4"/>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="6"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
@@ -2248,7 +2789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
@@ -2256,7 +2797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
@@ -2264,7 +2805,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
@@ -2272,7 +2813,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
@@ -2280,7 +2821,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
@@ -2288,7 +2829,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" s="7" t="s">
         <v>14</v>
       </c>
@@ -2296,7 +2837,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
@@ -2304,7 +2845,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" s="7" t="s">
         <v>18</v>
       </c>
@@ -2312,7 +2853,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" s="7" t="s">
         <v>20</v>
       </c>
@@ -2320,7 +2861,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14" s="7" t="s">
         <v>22</v>
       </c>
@@ -2328,17 +2869,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
     </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A16" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B16" s="9"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
         <v>25</v>
       </c>
@@ -2346,7 +2887,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
         <v>27</v>
       </c>
@@ -2354,7 +2895,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
         <v>29</v>
       </c>
@@ -2362,7 +2903,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
         <v>31</v>
       </c>
@@ -2370,7 +2911,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
         <v>33</v>
       </c>
@@ -2378,17 +2919,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
     </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A23" s="11" t="s">
         <v>35</v>
       </c>
       <c r="B23" s="12"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A24" s="13" t="s">
         <v>36</v>
       </c>
@@ -2396,7 +2937,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A25" s="13" t="s">
         <v>38</v>
       </c>
@@ -2404,7 +2945,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A26" s="13" t="s">
         <v>40</v>
       </c>
@@ -2412,7 +2953,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A27" s="13" t="s">
         <v>42</v>
       </c>
@@ -2420,7 +2961,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A28" s="13" t="s">
         <v>44</v>
       </c>
@@ -2428,7 +2969,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A29" s="13" t="s">
         <v>46</v>
       </c>
@@ -2436,7 +2977,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
     </row>
@@ -2452,24 +2993,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413306D3-ABEF-48D2-8F7E-A52637E5578F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFF57C40-AF55-489A-9972-769B4BC278AE}">
   <sheetPr>
     <tabColor rgb="FF0099FF"/>
   </sheetPr>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.69140625" customWidth="1"/>
+    <col min="2" max="2" width="38.69140625" customWidth="1"/>
+    <col min="3" max="3" width="20.69140625" customWidth="1"/>
+    <col min="4" max="4" width="25.69140625" customWidth="1"/>
+    <col min="5" max="5" width="12.69140625" customWidth="1"/>
+    <col min="6" max="7" width="13.69140625" customWidth="1"/>
+    <col min="8" max="8" width="22.69140625" customWidth="1"/>
+    <col min="9" max="9" width="14.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="38.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="14" t="s">
         <v>48</v>
       </c>
@@ -2498,7 +3039,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -2525,7 +3066,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -2552,7 +3093,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="15">
         <v>3</v>
       </c>
@@ -2579,7 +3120,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -2606,7 +3147,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="15">
         <v>5</v>
       </c>
@@ -2633,7 +3174,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -2660,7 +3201,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="15">
         <v>7</v>
       </c>
@@ -2687,7 +3228,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="17">
         <v>8</v>
       </c>
@@ -2714,7 +3255,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="15">
         <v>9</v>
       </c>
@@ -2741,7 +3282,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="17">
         <v>10</v>
       </c>
@@ -2768,7 +3309,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="15">
         <v>11</v>
       </c>
@@ -2795,7 +3336,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="17">
         <v>12</v>
       </c>
@@ -2822,7 +3363,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="15">
         <v>13</v>
       </c>
@@ -2849,7 +3390,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="17">
         <v>14</v>
       </c>
@@ -2876,7 +3417,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="15">
         <v>15</v>
       </c>
@@ -2903,7 +3444,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -2920,19 +3461,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E12A33F-042A-4A87-BB10-23B5DD062E71}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F3FE75A-3157-40DE-A909-B46D19702A1F}">
   <sheetPr>
     <tabColor rgb="FF47AD70"/>
   </sheetPr>
   <dimension ref="A1:I26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="8" width="9.7109375" customWidth="1"/>
-    <col min="9" max="9" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.69140625" customWidth="1"/>
+    <col min="2" max="8" width="9.69140625" customWidth="1"/>
+    <col min="9" max="9" width="30.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="40" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
         <v>123</v>
       </c>
@@ -2945,7 +3486,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A2" s="19" t="s">
         <v>124</v>
       </c>
@@ -2974,7 +3515,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3" s="20" t="s">
         <v>132</v>
       </c>
@@ -2987,7 +3528,7 @@
       <c r="H3" s="21"/>
       <c r="I3" s="21"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A4" s="22" t="s">
         <v>133</v>
       </c>
@@ -3006,7 +3547,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5" s="22" t="s">
         <v>136</v>
       </c>
@@ -3025,7 +3566,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6" s="22" t="s">
         <v>138</v>
       </c>
@@ -3040,7 +3581,7 @@
       <c r="H6" s="24"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
         <v>139</v>
       </c>
@@ -3059,7 +3600,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A8" s="25" t="s">
         <v>141</v>
       </c>
@@ -3072,7 +3613,7 @@
       <c r="H8" s="26"/>
       <c r="I8" s="26"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
         <v>142</v>
       </c>
@@ -3093,7 +3634,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A10" s="22" t="s">
         <v>144</v>
       </c>
@@ -3110,7 +3651,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>146</v>
       </c>
@@ -3125,7 +3666,7 @@
       <c r="H11" s="24"/>
       <c r="I11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A12" s="22" t="s">
         <v>147</v>
       </c>
@@ -3142,7 +3683,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A13" s="22" t="s">
         <v>149</v>
       </c>
@@ -3159,7 +3700,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A14" s="20" t="s">
         <v>151</v>
       </c>
@@ -3172,7 +3713,7 @@
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A15" s="22" t="s">
         <v>152</v>
       </c>
@@ -3187,7 +3728,7 @@
       <c r="H15" s="24"/>
       <c r="I15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A16" s="22" t="s">
         <v>153</v>
       </c>
@@ -3204,7 +3745,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="22" t="s">
         <v>155</v>
       </c>
@@ -3225,7 +3766,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="22" t="s">
         <v>157</v>
       </c>
@@ -3246,7 +3787,7 @@
       <c r="H18" s="24"/>
       <c r="I18" s="22"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="22" t="s">
         <v>158</v>
       </c>
@@ -3263,7 +3804,7 @@
       <c r="H19" s="24"/>
       <c r="I19" s="22"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="25" t="s">
         <v>159</v>
       </c>
@@ -3276,7 +3817,7 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="22" t="s">
         <v>160</v>
       </c>
@@ -3295,7 +3836,7 @@
       <c r="H21" s="24"/>
       <c r="I21" s="22"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="22" t="s">
         <v>161</v>
       </c>
@@ -3312,7 +3853,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="22" t="s">
         <v>163</v>
       </c>
@@ -3327,7 +3868,7 @@
       <c r="H23" s="24"/>
       <c r="I23" s="22"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A24" s="22" t="s">
         <v>164</v>
       </c>
@@ -3344,7 +3885,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A25" s="22" t="s">
         <v>166</v>
       </c>
@@ -3361,7 +3902,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -3385,22 +3926,22 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51B63414-1DD3-481A-92BB-EFA357B806D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118305BC-6B7F-44B4-9C5F-D6AF421DECB3}">
   <sheetPr>
     <tabColor rgb="FF0000FF"/>
   </sheetPr>
   <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="30.69140625" customWidth="1"/>
+    <col min="2" max="2" width="26.69140625" customWidth="1"/>
+    <col min="3" max="3" width="16.69140625" customWidth="1"/>
+    <col min="4" max="4" width="12.69140625" customWidth="1"/>
+    <col min="5" max="5" width="18.69140625" customWidth="1"/>
+    <col min="6" max="6" width="30.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="27" t="s">
         <v>168</v>
       </c>
@@ -3410,7 +3951,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="28" t="s">
         <v>169</v>
       </c>
@@ -3430,7 +3971,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="29" t="s">
         <v>174</v>
       </c>
@@ -3440,7 +3981,7 @@
       <c r="E3" s="30"/>
       <c r="F3" s="30"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>175</v>
       </c>
@@ -3460,7 +4001,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>178</v>
       </c>
@@ -3478,7 +4019,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>180</v>
       </c>
@@ -3498,7 +4039,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>183</v>
       </c>
@@ -3518,7 +4059,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="32" t="s">
         <v>186</v>
       </c>
@@ -3528,7 +4069,7 @@
       <c r="E8" s="33"/>
       <c r="F8" s="33"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>187</v>
       </c>
@@ -3548,7 +4089,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>190</v>
       </c>
@@ -3566,7 +4107,7 @@
       </c>
       <c r="F10" s="4"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>192</v>
       </c>
@@ -3586,7 +4127,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>195</v>
       </c>
@@ -3606,7 +4147,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>198</v>
       </c>
@@ -3626,7 +4167,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="29" t="s">
         <v>201</v>
       </c>
@@ -3636,7 +4177,7 @@
       <c r="E14" s="30"/>
       <c r="F14" s="30"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>202</v>
       </c>
@@ -3656,7 +4197,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>205</v>
       </c>
@@ -3676,7 +4217,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>208</v>
       </c>
@@ -3696,7 +4237,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="32" t="s">
         <v>211</v>
       </c>
@@ -3706,7 +4247,7 @@
       <c r="E18" s="33"/>
       <c r="F18" s="33"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>212</v>
       </c>
@@ -3726,7 +4267,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -3746,7 +4287,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>218</v>
       </c>
@@ -3766,7 +4307,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>221</v>
       </c>
@@ -3786,7 +4327,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="29" t="s">
         <v>224</v>
       </c>
@@ -3796,7 +4337,7 @@
       <c r="E23" s="30"/>
       <c r="F23" s="30"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>225</v>
       </c>
@@ -3816,7 +4357,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>228</v>
       </c>
@@ -3834,7 +4375,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>230</v>
       </c>
@@ -3854,7 +4395,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>233</v>
       </c>
@@ -3872,7 +4413,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="16.75" x14ac:dyDescent="0.45">
       <c r="A28" s="34" t="s">
         <v>235</v>
       </c>
@@ -3901,19 +4442,19 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{082BD061-E24A-4F42-8DAA-16D8C18EE7F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00797145-8D97-4F7B-8F53-2F1F7B7533AA}">
   <sheetPr>
     <tabColor rgb="FFA03070"/>
   </sheetPr>
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.69140625" customWidth="1"/>
+    <col min="2" max="6" width="14.69140625" customWidth="1"/>
+    <col min="7" max="7" width="28.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="38" t="s">
         <v>237</v>
       </c>
@@ -3924,7 +4465,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="39" t="s">
         <v>238</v>
       </c>
@@ -3947,7 +4488,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="40" t="s">
         <v>244</v>
       </c>
@@ -3958,7 +4499,7 @@
       <c r="F3" s="41"/>
       <c r="G3" s="41"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="42" t="s">
         <v>245</v>
       </c>
@@ -3981,7 +4522,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="44" t="s">
         <v>247</v>
       </c>
@@ -4002,7 +4543,7 @@
       </c>
       <c r="G5" s="44"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="42" t="s">
         <v>249</v>
       </c>
@@ -4025,7 +4566,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="44" t="s">
         <v>251</v>
       </c>
@@ -4048,7 +4589,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="40" t="s">
         <v>253</v>
       </c>
@@ -4059,7 +4600,7 @@
       <c r="F8" s="41"/>
       <c r="G8" s="41"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="44" t="s">
         <v>254</v>
       </c>
@@ -4082,7 +4623,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="42" t="s">
         <v>256</v>
       </c>
@@ -4105,7 +4646,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="44" t="s">
         <v>258</v>
       </c>
@@ -4126,7 +4667,7 @@
       </c>
       <c r="G11" s="44"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="42" t="s">
         <v>264</v>
       </c>
@@ -4147,7 +4688,7 @@
       </c>
       <c r="G12" s="42"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="44" t="s">
         <v>265</v>
       </c>
@@ -4170,7 +4711,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="42" t="s">
         <v>267</v>
       </c>
@@ -4193,7 +4734,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="40" t="s">
         <v>269</v>
       </c>
@@ -4204,7 +4745,7 @@
       <c r="F15" s="41"/>
       <c r="G15" s="41"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="42" t="s">
         <v>270</v>
       </c>
@@ -4227,7 +4768,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="44" t="s">
         <v>273</v>
       </c>
@@ -4250,7 +4791,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="42" t="s">
         <v>277</v>
       </c>
@@ -4271,7 +4812,7 @@
       </c>
       <c r="G18" s="42"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="40" t="s">
         <v>279</v>
       </c>
@@ -4282,7 +4823,7 @@
       <c r="F19" s="41"/>
       <c r="G19" s="41"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="42" t="s">
         <v>280</v>
       </c>
@@ -4305,7 +4846,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="44" t="s">
         <v>282</v>
       </c>
@@ -4328,7 +4869,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="42" t="s">
         <v>284</v>
       </c>
@@ -4351,7 +4892,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="40" t="s">
         <v>286</v>
       </c>
@@ -4362,7 +4903,7 @@
       <c r="F23" s="41"/>
       <c r="G23" s="41"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="42" t="s">
         <v>287</v>
       </c>
@@ -4385,7 +4926,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="44" t="s">
         <v>289</v>
       </c>
@@ -4408,7 +4949,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="42" t="s">
         <v>291</v>
       </c>
@@ -4431,7 +4972,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -4454,21 +4995,21 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D48C1AD3-38B6-4E3B-948E-F4DE388EFA1F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AC61631-2F34-48AC-99E8-7CDF3D7106F8}">
   <sheetPr>
     <tabColor rgb="FFF0B000"/>
   </sheetPr>
   <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.69140625" customWidth="1"/>
+    <col min="2" max="2" width="24.69140625" customWidth="1"/>
+    <col min="3" max="3" width="42.69140625" customWidth="1"/>
+    <col min="4" max="4" width="14.69140625" customWidth="1"/>
+    <col min="5" max="5" width="28.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="48" t="s">
         <v>293</v>
       </c>
@@ -4477,7 +5018,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="49" t="s">
         <v>294</v>
       </c>
@@ -4494,7 +5035,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="50">
         <v>1</v>
       </c>
@@ -4511,7 +5052,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="51"/>
       <c r="B4" s="51"/>
       <c r="C4" s="51" t="s">
@@ -4524,7 +5065,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="51"/>
       <c r="B5" s="51"/>
       <c r="C5" s="51" t="s">
@@ -4537,7 +5078,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="51"/>
       <c r="B6" s="51"/>
       <c r="C6" s="51" t="s">
@@ -4550,7 +5091,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="51"/>
       <c r="B7" s="51"/>
       <c r="C7" s="51" t="s">
@@ -4563,7 +5104,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="52">
         <v>2</v>
       </c>
@@ -4580,7 +5121,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16" t="s">
@@ -4593,7 +5134,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="16"/>
       <c r="B10" s="16"/>
       <c r="C10" s="16" t="s">
@@ -4606,7 +5147,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -4623,7 +5164,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="54"/>
       <c r="B12" s="54"/>
       <c r="C12" s="54" t="s">
@@ -4636,7 +5177,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="54"/>
       <c r="B13" s="54"/>
       <c r="C13" s="54" t="s">
@@ -4649,7 +5190,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="55">
         <v>4</v>
       </c>
@@ -4666,7 +5207,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="56"/>
       <c r="B15" s="56"/>
       <c r="C15" s="56" t="s">
@@ -4677,7 +5218,7 @@
       </c>
       <c r="E15" s="56"/>
     </row>
-    <row r="16" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="56"/>
       <c r="B16" s="56"/>
       <c r="C16" s="56" t="s">
@@ -4690,7 +5231,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="56"/>
       <c r="B17" s="56"/>
       <c r="C17" s="56" t="s">
@@ -4701,7 +5242,7 @@
       </c>
       <c r="E17" s="56"/>
     </row>
-    <row r="18" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="56"/>
       <c r="B18" s="56"/>
       <c r="C18" s="56" t="s">
@@ -4714,7 +5255,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="56"/>
       <c r="B19" s="56"/>
       <c r="C19" s="56" t="s">
@@ -4725,7 +5266,7 @@
       </c>
       <c r="E19" s="56"/>
     </row>
-    <row r="20" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="57">
         <v>5</v>
       </c>
@@ -4742,7 +5283,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="58"/>
       <c r="B21" s="58"/>
       <c r="C21" s="58" t="s">
@@ -4755,7 +5296,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="58"/>
       <c r="B22" s="58"/>
       <c r="C22" s="58" t="s">
@@ -4768,7 +5309,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="58"/>
       <c r="B23" s="58"/>
       <c r="C23" s="58" t="s">
@@ -4781,7 +5322,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="58"/>
       <c r="B24" s="58"/>
       <c r="C24" s="58" t="s">
@@ -4794,7 +5335,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="58"/>
       <c r="B25" s="58"/>
       <c r="C25" s="58" t="s">
@@ -4807,7 +5348,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="59">
         <v>6</v>
       </c>
@@ -4824,7 +5365,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="60"/>
       <c r="B27" s="60"/>
       <c r="C27" s="60" t="s">
@@ -4837,7 +5378,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="60"/>
       <c r="B28" s="60"/>
       <c r="C28" s="60" t="s">
@@ -4848,7 +5389,7 @@
       </c>
       <c r="E28" s="60"/>
     </row>
-    <row r="29" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="61">
         <v>7</v>
       </c>
@@ -4865,7 +5406,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="62"/>
       <c r="B30" s="62"/>
       <c r="C30" s="62" t="s">
@@ -4876,7 +5417,7 @@
       </c>
       <c r="E30" s="62"/>
     </row>
-    <row r="31" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="62"/>
       <c r="B31" s="62"/>
       <c r="C31" s="62" t="s">
@@ -4889,7 +5430,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="62"/>
       <c r="B32" s="62"/>
       <c r="C32" s="62" t="s">
@@ -4902,7 +5443,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4918,22 +5459,22 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E4976A1-C4F3-424F-A423-EC1563B887E6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0EB9D40-A180-4BB6-B959-8B4A804B1DBC}">
   <sheetPr>
     <tabColor rgb="FF9D6BFF"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.69140625" customWidth="1"/>
+    <col min="2" max="2" width="8.69140625" customWidth="1"/>
+    <col min="3" max="3" width="32.69140625" customWidth="1"/>
+    <col min="4" max="4" width="28.69140625" customWidth="1"/>
+    <col min="5" max="5" width="22.69140625" customWidth="1"/>
+    <col min="6" max="6" width="20.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="63" t="s">
         <v>370</v>
       </c>
@@ -4943,7 +5484,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="64" t="s">
         <v>371</v>
       </c>
@@ -4963,7 +5504,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="65" t="s">
         <v>377</v>
       </c>
@@ -4973,7 +5514,7 @@
       <c r="E3" s="66"/>
       <c r="F3" s="66"/>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="67" t="s">
         <v>378</v>
       </c>
@@ -4993,7 +5534,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="17" t="s">
         <v>378</v>
       </c>
@@ -5013,7 +5554,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="67" t="s">
         <v>378</v>
       </c>
@@ -5033,7 +5574,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="17" t="s">
         <v>378</v>
       </c>
@@ -5053,7 +5594,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="67" t="s">
         <v>378</v>
       </c>
@@ -5073,7 +5614,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="17" t="s">
         <v>378</v>
       </c>
@@ -5093,7 +5634,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="68" t="s">
         <v>409</v>
       </c>
@@ -5103,7 +5644,7 @@
       <c r="E10" s="69"/>
       <c r="F10" s="69"/>
     </row>
-    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="17" t="s">
         <v>410</v>
       </c>
@@ -5123,7 +5664,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="67" t="s">
         <v>410</v>
       </c>
@@ -5143,7 +5684,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="17" t="s">
         <v>410</v>
       </c>
@@ -5163,7 +5704,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="67" t="s">
         <v>410</v>
       </c>
@@ -5183,7 +5724,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="17" t="s">
         <v>410</v>
       </c>
@@ -5203,7 +5744,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="67" t="s">
         <v>410</v>
       </c>
@@ -5223,7 +5764,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="70" t="s">
         <v>433</v>
       </c>
@@ -5233,7 +5774,7 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="67" t="s">
         <v>434</v>
       </c>
@@ -5253,7 +5794,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="17" t="s">
         <v>434</v>
       </c>
@@ -5273,7 +5814,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="67" t="s">
         <v>434</v>
       </c>
@@ -5293,7 +5834,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="17" t="s">
         <v>434</v>
       </c>
@@ -5313,7 +5854,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="67" t="s">
         <v>434</v>
       </c>
@@ -5333,7 +5874,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="17" t="s">
         <v>434</v>
       </c>
@@ -5353,7 +5894,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="71" t="s">
         <v>458</v>
       </c>
@@ -5363,7 +5904,7 @@
       <c r="E24" s="72"/>
       <c r="F24" s="72"/>
     </row>
-    <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="17" t="s">
         <v>459</v>
       </c>
@@ -5383,7 +5924,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="67" t="s">
         <v>459</v>
       </c>
@@ -5403,7 +5944,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="17" t="s">
         <v>459</v>
       </c>
@@ -5423,7 +5964,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="67" t="s">
         <v>459</v>
       </c>
@@ -5443,7 +5984,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -5461,4 +6002,812 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{035F98B8-038F-423A-BD37-88F6F5272949}">
+  <sheetPr>
+    <tabColor rgb="FF50B000"/>
+  </sheetPr>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="8.69140625" customWidth="1"/>
+    <col min="2" max="2" width="20.69140625" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" customWidth="1"/>
+    <col min="4" max="4" width="28.69140625" customWidth="1"/>
+    <col min="5" max="5" width="16.69140625" customWidth="1"/>
+    <col min="6" max="6" width="14.69140625" customWidth="1"/>
+    <col min="7" max="7" width="26.69140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="73" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="74" t="s">
+        <v>294</v>
+      </c>
+      <c r="B2" s="74" t="s">
+        <v>476</v>
+      </c>
+      <c r="C2" s="74" t="s">
+        <v>477</v>
+      </c>
+      <c r="D2" s="74" t="s">
+        <v>478</v>
+      </c>
+      <c r="E2" s="74" t="s">
+        <v>479</v>
+      </c>
+      <c r="F2" s="74" t="s">
+        <v>480</v>
+      </c>
+      <c r="G2" s="74" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="75" t="s">
+        <v>482</v>
+      </c>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+    </row>
+    <row r="4" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="77">
+        <v>1</v>
+      </c>
+      <c r="B4" s="77" t="s">
+        <v>483</v>
+      </c>
+      <c r="C4" s="77" t="s">
+        <v>484</v>
+      </c>
+      <c r="D4" s="77" t="s">
+        <v>485</v>
+      </c>
+      <c r="E4" s="77" t="s">
+        <v>486</v>
+      </c>
+      <c r="F4" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G4" s="77" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="17">
+        <v>1</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>489</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>491</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="F5" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="77">
+        <v>1</v>
+      </c>
+      <c r="B6" s="77" t="s">
+        <v>495</v>
+      </c>
+      <c r="C6" s="77" t="s">
+        <v>496</v>
+      </c>
+      <c r="D6" s="77" t="s">
+        <v>497</v>
+      </c>
+      <c r="E6" s="77" t="s">
+        <v>498</v>
+      </c>
+      <c r="F6" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G6" s="77" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="81" t="s">
+        <v>501</v>
+      </c>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
+      <c r="G7" s="82"/>
+    </row>
+    <row r="8" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="77">
+        <v>2</v>
+      </c>
+      <c r="B8" s="77" t="s">
+        <v>502</v>
+      </c>
+      <c r="C8" s="77" t="s">
+        <v>503</v>
+      </c>
+      <c r="D8" s="77" t="s">
+        <v>504</v>
+      </c>
+      <c r="E8" s="77" t="s">
+        <v>505</v>
+      </c>
+      <c r="F8" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G8" s="77" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="17">
+        <v>2</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>507</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>508</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>509</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>510</v>
+      </c>
+      <c r="F9" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="77">
+        <v>2</v>
+      </c>
+      <c r="B10" s="77" t="s">
+        <v>512</v>
+      </c>
+      <c r="C10" s="77" t="s">
+        <v>513</v>
+      </c>
+      <c r="D10" s="77" t="s">
+        <v>514</v>
+      </c>
+      <c r="E10" s="77" t="s">
+        <v>515</v>
+      </c>
+      <c r="F10" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G10" s="77" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="17">
+        <v>2</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>517</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>486</v>
+      </c>
+      <c r="F11" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="83" t="s">
+        <v>521</v>
+      </c>
+      <c r="B12" s="84"/>
+      <c r="C12" s="84"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
+    </row>
+    <row r="13" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="17">
+        <v>3</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>522</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>523</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>524</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="F13" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="77">
+        <v>3</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>527</v>
+      </c>
+      <c r="C14" s="77" t="s">
+        <v>528</v>
+      </c>
+      <c r="D14" s="77" t="s">
+        <v>529</v>
+      </c>
+      <c r="E14" s="77" t="s">
+        <v>530</v>
+      </c>
+      <c r="F14" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G14" s="77" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="17">
+        <v>3</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>532</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>533</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="F15" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="77">
+        <v>3</v>
+      </c>
+      <c r="B16" s="77" t="s">
+        <v>536</v>
+      </c>
+      <c r="C16" s="77" t="s">
+        <v>537</v>
+      </c>
+      <c r="D16" s="77" t="s">
+        <v>538</v>
+      </c>
+      <c r="E16" s="77" t="s">
+        <v>486</v>
+      </c>
+      <c r="F16" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G16" s="77" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="17">
+        <v>3</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>540</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>541</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F17" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="85" t="s">
+        <v>545</v>
+      </c>
+      <c r="B18" s="86"/>
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="86"/>
+      <c r="G18" s="86"/>
+    </row>
+    <row r="19" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="17">
+        <v>4</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>546</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>547</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>548</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="F19" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="77">
+        <v>4</v>
+      </c>
+      <c r="B20" s="77" t="s">
+        <v>551</v>
+      </c>
+      <c r="C20" s="77" t="s">
+        <v>552</v>
+      </c>
+      <c r="D20" s="77" t="s">
+        <v>553</v>
+      </c>
+      <c r="E20" s="77" t="s">
+        <v>525</v>
+      </c>
+      <c r="F20" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G20" s="77" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="17">
+        <v>4</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>555</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>556</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="F21" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="77">
+        <v>4</v>
+      </c>
+      <c r="B22" s="77" t="s">
+        <v>560</v>
+      </c>
+      <c r="C22" s="77" t="s">
+        <v>561</v>
+      </c>
+      <c r="D22" s="77" t="s">
+        <v>562</v>
+      </c>
+      <c r="E22" s="77" t="s">
+        <v>505</v>
+      </c>
+      <c r="F22" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G22" s="77" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="17">
+        <v>4</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>564</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>565</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="F23" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="87" t="s">
+        <v>568</v>
+      </c>
+      <c r="B24" s="88"/>
+      <c r="C24" s="88"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="88"/>
+    </row>
+    <row r="25" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="17">
+        <v>5</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>569</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>570</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>486</v>
+      </c>
+      <c r="F25" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="77">
+        <v>5</v>
+      </c>
+      <c r="B26" s="77" t="s">
+        <v>573</v>
+      </c>
+      <c r="C26" s="77" t="s">
+        <v>574</v>
+      </c>
+      <c r="D26" s="77" t="s">
+        <v>575</v>
+      </c>
+      <c r="E26" s="77" t="s">
+        <v>505</v>
+      </c>
+      <c r="F26" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G26" s="77" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="17">
+        <v>5</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>577</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>578</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>579</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="F27" s="89" t="s">
+        <v>580</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="90" t="s">
+        <v>582</v>
+      </c>
+      <c r="B28" s="91"/>
+      <c r="C28" s="91"/>
+      <c r="D28" s="91"/>
+      <c r="E28" s="91"/>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91"/>
+    </row>
+    <row r="29" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="17">
+        <v>6</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>583</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>584</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>585</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>486</v>
+      </c>
+      <c r="F29" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="77">
+        <v>6</v>
+      </c>
+      <c r="B30" s="77" t="s">
+        <v>587</v>
+      </c>
+      <c r="C30" s="77" t="s">
+        <v>588</v>
+      </c>
+      <c r="D30" s="77" t="s">
+        <v>589</v>
+      </c>
+      <c r="E30" s="77" t="s">
+        <v>486</v>
+      </c>
+      <c r="F30" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G30" s="77" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="17">
+        <v>6</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>591</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>592</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="F31" s="78" t="s">
+        <v>487</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="77">
+        <v>6</v>
+      </c>
+      <c r="B32" s="77" t="s">
+        <v>595</v>
+      </c>
+      <c r="C32" s="77" t="s">
+        <v>596</v>
+      </c>
+      <c r="D32" s="77" t="s">
+        <v>597</v>
+      </c>
+      <c r="E32" s="77" t="s">
+        <v>492</v>
+      </c>
+      <c r="F32" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G32" s="77" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="83" t="s">
+        <v>599</v>
+      </c>
+      <c r="B33" s="84"/>
+      <c r="C33" s="84"/>
+      <c r="D33" s="84"/>
+      <c r="E33" s="84"/>
+      <c r="F33" s="84"/>
+      <c r="G33" s="84"/>
+    </row>
+    <row r="34" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="77">
+        <v>7</v>
+      </c>
+      <c r="B34" s="77" t="s">
+        <v>600</v>
+      </c>
+      <c r="C34" s="77" t="s">
+        <v>601</v>
+      </c>
+      <c r="D34" s="77" t="s">
+        <v>602</v>
+      </c>
+      <c r="E34" s="77" t="s">
+        <v>492</v>
+      </c>
+      <c r="F34" s="89" t="s">
+        <v>580</v>
+      </c>
+      <c r="G34" s="77" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="17">
+        <v>7</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>604</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>605</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>606</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="F35" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="77">
+        <v>7</v>
+      </c>
+      <c r="B36" s="77" t="s">
+        <v>608</v>
+      </c>
+      <c r="C36" s="77" t="s">
+        <v>609</v>
+      </c>
+      <c r="D36" s="77" t="s">
+        <v>610</v>
+      </c>
+      <c r="E36" s="77" t="s">
+        <v>505</v>
+      </c>
+      <c r="F36" s="80" t="s">
+        <v>499</v>
+      </c>
+      <c r="G36" s="77" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="17">
+        <v>7</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>613</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>614</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="F37" s="79" t="s">
+        <v>493</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+    </row>
+    <row r="39" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="92" t="s">
+        <v>616</v>
+      </c>
+      <c r="B39" s="93"/>
+      <c r="C39" s="93"/>
+      <c r="D39" s="93"/>
+      <c r="E39" s="93"/>
+      <c r="F39" s="93"/>
+      <c r="G39" s="93"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A24:G24"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>